<commit_message>
update results with elected reps
</commit_message>
<xml_diff>
--- a/src/data/raw/adjara_2008_candidates.xlsx
+++ b/src/data/raw/adjara_2008_candidates.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox (Personal)\My projects\Elections\Results\2008_adjara\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox (Personal)\My projects\Elections\ge_elections_dashboard\wireframe\observable_framework\elections_data\src\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACBF936-5E2E-45D9-A61E-9A997F1FC3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE2E7C1-86BE-4299-A8F4-56E3D8683529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2442,82 +2442,82 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B6" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
@@ -2528,44 +2528,44 @@
         <v>0</v>
       </c>
       <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
         <v>7</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -2574,70 +2574,70 @@
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B10" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B11" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E11" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="F11" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
@@ -2648,84 +2648,84 @@
         <v>1</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F13" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E15" t="s">
         <v>48</v>
       </c>
       <c r="F15" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B16" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E16" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="F16" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B17" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C17">
         <v>3</v>
@@ -2734,18 +2734,18 @@
         <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B18" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C18">
         <v>4</v>
@@ -2754,10 +2754,10 @@
         <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="F18" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.4">
@@ -2768,96 +2768,96 @@
         <v>2</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E19" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F19" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B20" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="F20" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B21" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C21">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="F21" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B22" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F22" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B23" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D23" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F23" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.4">
@@ -2868,24 +2868,24 @@
         <v>3</v>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E24" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="F24" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B25" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25">
         <v>5</v>
@@ -2894,190 +2894,190 @@
         <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="F25" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B26" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C26">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="F26" t="s">
-        <v>29</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B27" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C27">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D27" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E27" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="F27" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B28" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C28">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E28" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="F28" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B29" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D29" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E29" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F29" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B30" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C30">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D30" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E30" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="F30" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C31">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="F31" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B32" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C32">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="F32" t="s">
-        <v>77</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B33" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C33">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="F33" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B34" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C34">
         <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F34" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.4">
@@ -3088,16 +3088,16 @@
         <v>4</v>
       </c>
       <c r="C35">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F35" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.4">
@@ -3108,13 +3108,13 @@
         <v>5</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="F36" t="s">
         <v>82</v>
@@ -3122,102 +3122,102 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C37">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D37" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="F37" t="s">
-        <v>83</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B38" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C38">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="F38" t="s">
-        <v>85</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C39">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D39" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C40">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D40" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="F40" t="s">
-        <v>89</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B41" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C41">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D41" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F41" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.4">
@@ -3241,6 +3241,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F42">
+    <sortCondition ref="C2:C42"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>